<commit_message>
Mise à jour site
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\platres-et-enduits\prix\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caisse5\Desktop\site-internet\platres-et-enduits\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A489E4-36FD-449E-9EDE-2F9001742A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36A36D4D-891B-49DF-9424-0B93C11DDE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11016" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="409">
   <si>
     <t>path</t>
   </si>
@@ -1036,6 +1036,252 @@
   </si>
   <si>
     <t>galerie/vis-montage-rapide-pfs.png</t>
+  </si>
+  <si>
+    <t>61063472</t>
+  </si>
+  <si>
+    <t>61063474</t>
+  </si>
+  <si>
+    <t>61063475</t>
+  </si>
+  <si>
+    <t>61063476</t>
+  </si>
+  <si>
+    <t>61063477</t>
+  </si>
+  <si>
+    <t>61063480</t>
+  </si>
+  <si>
+    <t>61063484</t>
+  </si>
+  <si>
+    <t>61063486</t>
+  </si>
+  <si>
+    <t>61063488</t>
+  </si>
+  <si>
+    <t>61063492</t>
+  </si>
+  <si>
+    <t>61063494</t>
+  </si>
+  <si>
+    <t>Platresse INOX  280</t>
+  </si>
+  <si>
+    <t>Platresse INOX  260 mm cp217426</t>
+  </si>
+  <si>
+    <t>Platresse a chape cp400262</t>
+  </si>
+  <si>
+    <t>Platresse inox- 0.3mm 28x11</t>
+  </si>
+  <si>
+    <t>Platresse inox- 0.3mm 35X11</t>
+  </si>
+  <si>
+    <t>Platresse ACIER 280</t>
+  </si>
+  <si>
+    <t>Platresse  inox 280 mm dent 6 x 6 m</t>
+  </si>
+  <si>
+    <t>Platresse inox 280 mm dent 8 x 8 mm</t>
+  </si>
+  <si>
+    <t>Platresse inox 280 mm dent 10 x 10</t>
+  </si>
+  <si>
+    <t>Platresse inox 100x450 arrondie</t>
+  </si>
+  <si>
+    <t>Platresse inox 120x305 arrondie 0.65</t>
+  </si>
+  <si>
+    <t>61118599</t>
+  </si>
+  <si>
+    <t>61118606</t>
+  </si>
+  <si>
+    <t>61118607</t>
+  </si>
+  <si>
+    <t>61118610</t>
+  </si>
+  <si>
+    <t>61118611</t>
+  </si>
+  <si>
+    <t>61118612</t>
+  </si>
+  <si>
+    <t>61118614</t>
+  </si>
+  <si>
+    <t>61118651</t>
+  </si>
+  <si>
+    <t>61118652</t>
+  </si>
+  <si>
+    <t>61119013</t>
+  </si>
+  <si>
+    <t>61119014</t>
+  </si>
+  <si>
+    <t>61119015</t>
+  </si>
+  <si>
+    <t>61119022</t>
+  </si>
+  <si>
+    <t>61119180</t>
+  </si>
+  <si>
+    <t>61119182</t>
+  </si>
+  <si>
+    <t>61119184</t>
+  </si>
+  <si>
+    <t>61119190</t>
+  </si>
+  <si>
+    <t>61119191</t>
+  </si>
+  <si>
+    <t>61119192</t>
+  </si>
+  <si>
+    <t>61119196</t>
+  </si>
+  <si>
+    <t>61119198</t>
+  </si>
+  <si>
+    <t>61119200</t>
+  </si>
+  <si>
+    <t>611192000</t>
+  </si>
+  <si>
+    <t>61119201</t>
+  </si>
+  <si>
+    <t>61119202</t>
+  </si>
+  <si>
+    <t>61119204</t>
+  </si>
+  <si>
+    <t>61119206</t>
+  </si>
+  <si>
+    <t>61119210</t>
+  </si>
+  <si>
+    <t>platress+B2:B26e inox 280x130mm</t>
+  </si>
+  <si>
+    <t>Platresse  hollande dentée inox 33433440</t>
+  </si>
+  <si>
+    <t>Platresse  hollande dentée inoxx</t>
+  </si>
+  <si>
+    <t>Platresse hollande inox 28x13 33433437</t>
+  </si>
+  <si>
+    <t>Palette de platrier alu ds36950</t>
+  </si>
+  <si>
+    <t>Platresse inox dentee 12x12</t>
+  </si>
+  <si>
+    <t>Platresse acier pointue 110x400</t>
+  </si>
+  <si>
+    <t>Platresse Plasticflex 330x110x1mm</t>
+  </si>
+  <si>
+    <t>Platresse coins arrondis 406x100</t>
+  </si>
+  <si>
+    <t>Taloche plastique 14x8cm</t>
+  </si>
+  <si>
+    <t>Taloche gratton 14x24cm</t>
+  </si>
+  <si>
+    <t>Taloche frottoir blanc 120x250</t>
+  </si>
+  <si>
+    <t>Trepan multi mat.D35</t>
+  </si>
+  <si>
+    <t>Palette de joint droite - inox 230</t>
+  </si>
+  <si>
+    <t>Palette de joint gauche - inox 230</t>
+  </si>
+  <si>
+    <t>Palette de joint droite pl252132</t>
+  </si>
+  <si>
+    <t>Taloche point polyst noir 27x18</t>
+  </si>
+  <si>
+    <t>Taloche point polyst noir  27x18</t>
+  </si>
+  <si>
+    <t>Taloche rect polyst noir 350 x 260m</t>
+  </si>
+  <si>
+    <t>Taloche rect. épong oran. pl260028</t>
+  </si>
+  <si>
+    <t>Taloche angulaire éponge orange</t>
+  </si>
+  <si>
+    <t>Taloche éponge orange</t>
+  </si>
+  <si>
+    <t>Taloche mousse orange</t>
+  </si>
+  <si>
+    <t>Taloche éponge noire</t>
+  </si>
+  <si>
+    <t>Frottoir en polyurethane 280x140</t>
+  </si>
+  <si>
+    <t>Platoir ragni 318 28x12</t>
+  </si>
+  <si>
+    <t>Platoir plast semelle hydro eponge</t>
+  </si>
+  <si>
+    <t>Platoir plast rape métal 108127</t>
+  </si>
+  <si>
+    <t>61063286</t>
+  </si>
+  <si>
+    <t>61063287</t>
+  </si>
+  <si>
+    <t>Couteau à enduire 800mm x 0.3mm</t>
+  </si>
+  <si>
+    <t>Couteau à enduire 600mm x 0.3mm</t>
   </si>
 </sst>
 </file>
@@ -1171,7 +1417,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1204,17 +1450,11 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1228,24 +1468,21 @@
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1601,7 +1838,7 @@
       <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="18" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
@@ -1656,7 +1893,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="25"/>
+      <c r="A4" s="20"/>
       <c r="B4" s="11" t="s">
         <v>71</v>
       </c>
@@ -1674,7 +1911,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="25"/>
+      <c r="A5" s="20"/>
       <c r="B5" s="11" t="s">
         <v>72</v>
       </c>
@@ -1792,7 +2029,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="25"/>
+      <c r="A11" s="20"/>
       <c r="B11" s="11" t="s">
         <v>78</v>
       </c>
@@ -1850,7 +2087,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="25"/>
+      <c r="A14" s="20"/>
       <c r="B14" s="2" t="s">
         <v>321</v>
       </c>
@@ -2008,7 +2245,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="25"/>
+      <c r="A22" s="20"/>
       <c r="B22" s="11" t="s">
         <v>88</v>
       </c>
@@ -2026,7 +2263,7 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="25"/>
+      <c r="A23" s="20"/>
       <c r="B23" s="11" t="s">
         <v>89</v>
       </c>
@@ -2044,7 +2281,7 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="25"/>
+      <c r="A24" s="20"/>
       <c r="B24" s="11" t="s">
         <v>90</v>
       </c>
@@ -2062,7 +2299,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="25"/>
+      <c r="A25" s="20"/>
       <c r="B25" s="11" t="s">
         <v>91</v>
       </c>
@@ -2160,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="25"/>
+      <c r="A30" s="20"/>
       <c r="B30" s="11" t="s">
         <v>96</v>
       </c>
@@ -2178,7 +2415,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="25"/>
+      <c r="A31" s="20"/>
       <c r="B31" s="11" t="s">
         <v>97</v>
       </c>
@@ -2216,7 +2453,7 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="25"/>
+      <c r="A33" s="20"/>
       <c r="B33" s="11" t="s">
         <v>99</v>
       </c>
@@ -2234,7 +2471,7 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="25"/>
+      <c r="A34" s="20"/>
       <c r="B34" s="11" t="s">
         <v>100</v>
       </c>
@@ -2252,7 +2489,7 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="25"/>
+      <c r="A35" s="20"/>
       <c r="B35" s="11" t="s">
         <v>101</v>
       </c>
@@ -2270,7 +2507,7 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="25"/>
+      <c r="A36" s="20"/>
       <c r="B36" s="11" t="s">
         <v>102</v>
       </c>
@@ -2351,7 +2588,7 @@
       <c r="A40" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="B40" s="16" t="s">
+      <c r="B40" s="14" t="s">
         <v>19</v>
       </c>
       <c r="C40" s="5" t="s">
@@ -2420,7 +2657,7 @@
       <c r="D43" s="3">
         <v>20.76</v>
       </c>
-      <c r="E43" s="17" t="s">
+      <c r="E43" s="15" t="s">
         <v>12</v>
       </c>
       <c r="F43" s="5">
@@ -2440,7 +2677,7 @@
       <c r="D44" s="3">
         <v>31.470000000000002</v>
       </c>
-      <c r="E44" s="17" t="s">
+      <c r="E44" s="15" t="s">
         <v>13</v>
       </c>
       <c r="F44" s="5">
@@ -2460,7 +2697,7 @@
       <c r="D45" s="3">
         <v>21.89</v>
       </c>
-      <c r="E45" s="18" t="s">
+      <c r="E45" s="16" t="s">
         <v>14</v>
       </c>
       <c r="F45" s="5">
@@ -2480,7 +2717,7 @@
       <c r="D46" s="3">
         <v>6.6400000000000006</v>
       </c>
-      <c r="E46" s="18" t="s">
+      <c r="E46" s="16" t="s">
         <v>15</v>
       </c>
       <c r="F46" s="5">
@@ -2500,7 +2737,7 @@
       <c r="D47" s="3">
         <v>5.47</v>
       </c>
-      <c r="E47" s="19" t="s">
+      <c r="E47" s="17" t="s">
         <v>103</v>
       </c>
       <c r="F47" s="5">
@@ -2520,7 +2757,7 @@
       <c r="D48" s="3">
         <v>4.33</v>
       </c>
-      <c r="E48" s="19" t="s">
+      <c r="E48" s="17" t="s">
         <v>104</v>
       </c>
       <c r="F48" s="5">
@@ -2540,7 +2777,7 @@
       <c r="D49" s="3">
         <v>4.84</v>
       </c>
-      <c r="E49" s="19" t="s">
+      <c r="E49" s="17" t="s">
         <v>105</v>
       </c>
       <c r="F49" s="5">
@@ -2560,7 +2797,7 @@
       <c r="D50" s="3">
         <v>5.09</v>
       </c>
-      <c r="E50" s="19" t="s">
+      <c r="E50" s="17" t="s">
         <v>106</v>
       </c>
       <c r="F50" s="5">
@@ -2580,7 +2817,7 @@
       <c r="D51" s="3">
         <v>5.26</v>
       </c>
-      <c r="E51" s="19" t="s">
+      <c r="E51" s="17" t="s">
         <v>107</v>
       </c>
       <c r="F51" s="5">
@@ -2600,7 +2837,7 @@
       <c r="D52" s="3">
         <v>5.09</v>
       </c>
-      <c r="E52" s="19" t="s">
+      <c r="E52" s="17" t="s">
         <v>108</v>
       </c>
       <c r="F52" s="5">
@@ -2620,7 +2857,7 @@
       <c r="D53" s="3">
         <v>5.26</v>
       </c>
-      <c r="E53" s="19" t="s">
+      <c r="E53" s="17" t="s">
         <v>109</v>
       </c>
       <c r="F53" s="5">
@@ -2640,7 +2877,7 @@
       <c r="D54" s="3">
         <v>5.13</v>
       </c>
-      <c r="E54" s="19" t="s">
+      <c r="E54" s="17" t="s">
         <v>110</v>
       </c>
       <c r="F54" s="5">
@@ -2660,7 +2897,7 @@
       <c r="D55" s="3">
         <v>5.09</v>
       </c>
-      <c r="E55" s="19" t="s">
+      <c r="E55" s="17" t="s">
         <v>111</v>
       </c>
       <c r="F55" s="5">
@@ -2680,7 +2917,7 @@
       <c r="D56" s="3">
         <v>9.0400000000000009</v>
       </c>
-      <c r="E56" s="19" t="s">
+      <c r="E56" s="17" t="s">
         <v>112</v>
       </c>
       <c r="F56" s="5">
@@ -2700,7 +2937,7 @@
       <c r="D57" s="3">
         <v>9.0400000000000009</v>
       </c>
-      <c r="E57" s="19" t="s">
+      <c r="E57" s="17" t="s">
         <v>113</v>
       </c>
       <c r="F57" s="5">
@@ -2720,7 +2957,7 @@
       <c r="D58" s="3">
         <v>7.25</v>
       </c>
-      <c r="E58" s="19" t="s">
+      <c r="E58" s="17" t="s">
         <v>114</v>
       </c>
       <c r="F58" s="5">
@@ -2740,7 +2977,7 @@
       <c r="D59" s="3">
         <v>8.16</v>
       </c>
-      <c r="E59" s="19" t="s">
+      <c r="E59" s="17" t="s">
         <v>115</v>
       </c>
       <c r="F59" s="5">
@@ -2760,7 +2997,7 @@
       <c r="D60" s="3">
         <v>7.71</v>
       </c>
-      <c r="E60" s="19" t="s">
+      <c r="E60" s="17" t="s">
         <v>116</v>
       </c>
       <c r="F60" s="5">
@@ -2780,7 +3017,7 @@
       <c r="D61" s="3">
         <v>8.4499999999999993</v>
       </c>
-      <c r="E61" s="19" t="s">
+      <c r="E61" s="17" t="s">
         <v>117</v>
       </c>
       <c r="F61" s="5">
@@ -2791,7 +3028,7 @@
       <c r="A62" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="B62" s="16" t="s">
+      <c r="B62" s="14" t="s">
         <v>134</v>
       </c>
       <c r="C62" s="2" t="s">
@@ -2800,7 +3037,7 @@
       <c r="D62" s="3">
         <v>9.33</v>
       </c>
-      <c r="E62" s="19" t="s">
+      <c r="E62" s="17" t="s">
         <v>118</v>
       </c>
       <c r="F62" s="5">
@@ -2820,7 +3057,7 @@
       <c r="D63" s="3">
         <v>23.900000000000002</v>
       </c>
-      <c r="E63" s="20" t="s">
+      <c r="E63" s="22" t="s">
         <v>135</v>
       </c>
       <c r="F63" s="5">
@@ -2831,7 +3068,7 @@
       <c r="A64" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="B64" s="16" t="s">
+      <c r="B64" s="14" t="s">
         <v>144</v>
       </c>
       <c r="C64" s="2" t="s">
@@ -2840,7 +3077,7 @@
       <c r="D64" s="3">
         <v>10.9</v>
       </c>
-      <c r="E64" s="20" t="s">
+      <c r="E64" s="22" t="s">
         <v>136</v>
       </c>
       <c r="F64" s="5">
@@ -2860,7 +3097,7 @@
       <c r="D65" s="3">
         <v>12.06</v>
       </c>
-      <c r="E65" s="20" t="s">
+      <c r="E65" s="22" t="s">
         <v>137</v>
       </c>
       <c r="F65" s="5">
@@ -2880,7 +3117,7 @@
       <c r="D66" s="3">
         <v>1.78</v>
       </c>
-      <c r="E66" s="20" t="s">
+      <c r="E66" s="22" t="s">
         <v>138</v>
       </c>
       <c r="F66" s="5">
@@ -2900,7 +3137,7 @@
       <c r="D67" s="3">
         <v>5.48</v>
       </c>
-      <c r="E67" s="20" t="s">
+      <c r="E67" s="22" t="s">
         <v>139</v>
       </c>
       <c r="F67" s="5">
@@ -2908,7 +3145,7 @@
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A68" s="25"/>
+      <c r="A68" s="20"/>
       <c r="B68" s="11" t="s">
         <v>148</v>
       </c>
@@ -2918,7 +3155,7 @@
       <c r="D68" s="3">
         <v>5</v>
       </c>
-      <c r="E68" s="20" t="s">
+      <c r="E68" s="22" t="s">
         <v>140</v>
       </c>
       <c r="F68" s="5">
@@ -2938,7 +3175,7 @@
       <c r="D69" s="3">
         <v>5.49</v>
       </c>
-      <c r="E69" s="20" t="s">
+      <c r="E69" s="22" t="s">
         <v>141</v>
       </c>
       <c r="F69" s="5">
@@ -2946,7 +3183,7 @@
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A70" s="25"/>
+      <c r="A70" s="20"/>
       <c r="B70" s="11" t="s">
         <v>150</v>
       </c>
@@ -2956,7 +3193,7 @@
       <c r="D70" s="3">
         <v>19.41</v>
       </c>
-      <c r="E70" s="20" t="s">
+      <c r="E70" s="22" t="s">
         <v>142</v>
       </c>
       <c r="F70" s="5">
@@ -2976,13 +3213,13 @@
       <c r="D71" s="3">
         <v>25.8</v>
       </c>
-      <c r="E71" s="22" t="s">
+      <c r="E71" s="23" t="s">
         <v>151</v>
       </c>
       <c r="F71" s="5">
         <v>4</v>
       </c>
-      <c r="G71" s="23"/>
+      <c r="G71" s="19"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
@@ -2997,7 +3234,7 @@
       <c r="D72" s="3">
         <v>27.3</v>
       </c>
-      <c r="E72" s="22" t="s">
+      <c r="E72" s="23" t="s">
         <v>152</v>
       </c>
       <c r="F72" s="5">
@@ -3017,7 +3254,7 @@
       <c r="D73" s="3">
         <v>40.119999999999997</v>
       </c>
-      <c r="E73" s="22" t="s">
+      <c r="E73" s="23" t="s">
         <v>153</v>
       </c>
       <c r="F73" s="5">
@@ -3037,7 +3274,7 @@
       <c r="D74" s="3">
         <v>16.170000000000002</v>
       </c>
-      <c r="E74" s="22" t="s">
+      <c r="E74" s="23" t="s">
         <v>154</v>
       </c>
       <c r="F74" s="5">
@@ -3057,7 +3294,7 @@
       <c r="D75" s="3">
         <v>22.05</v>
       </c>
-      <c r="E75" s="22" t="s">
+      <c r="E75" s="23" t="s">
         <v>155</v>
       </c>
       <c r="F75" s="5">
@@ -3077,7 +3314,7 @@
       <c r="D76" s="3">
         <v>25.810000000000002</v>
       </c>
-      <c r="E76" s="22" t="s">
+      <c r="E76" s="23" t="s">
         <v>156</v>
       </c>
       <c r="F76" s="5">
@@ -3097,7 +3334,7 @@
       <c r="D77" s="3">
         <v>13.07</v>
       </c>
-      <c r="E77" s="22" t="s">
+      <c r="E77" s="23" t="s">
         <v>157</v>
       </c>
       <c r="F77" s="5">
@@ -3117,7 +3354,7 @@
       <c r="D78" s="3">
         <v>3.15</v>
       </c>
-      <c r="E78" s="22" t="s">
+      <c r="E78" s="23" t="s">
         <v>158</v>
       </c>
       <c r="F78" s="5">
@@ -3137,7 +3374,7 @@
       <c r="D79" s="3">
         <v>16.63</v>
       </c>
-      <c r="E79" s="22" t="s">
+      <c r="E79" s="23" t="s">
         <v>159</v>
       </c>
       <c r="F79" s="5">
@@ -3157,7 +3394,7 @@
       <c r="D80" s="3">
         <v>6.17</v>
       </c>
-      <c r="E80" s="22" t="s">
+      <c r="E80" s="23" t="s">
         <v>160</v>
       </c>
       <c r="F80" s="5">
@@ -3177,7 +3414,7 @@
       <c r="D81" s="3">
         <v>15.73</v>
       </c>
-      <c r="E81" s="22" t="s">
+      <c r="E81" s="23" t="s">
         <v>161</v>
       </c>
       <c r="F81" s="5">
@@ -3197,7 +3434,7 @@
       <c r="D82" s="3">
         <v>3.92</v>
       </c>
-      <c r="E82" s="22" t="s">
+      <c r="E82" s="23" t="s">
         <v>162</v>
       </c>
       <c r="F82" s="5">
@@ -3217,7 +3454,7 @@
       <c r="D83" s="3">
         <v>21.95</v>
       </c>
-      <c r="E83" s="22" t="s">
+      <c r="E83" s="23" t="s">
         <v>163</v>
       </c>
       <c r="F83" s="5">
@@ -3237,7 +3474,7 @@
       <c r="D84" s="3">
         <v>4.99</v>
       </c>
-      <c r="E84" s="22" t="s">
+      <c r="E84" s="23" t="s">
         <v>164</v>
       </c>
       <c r="F84" s="5">
@@ -3257,7 +3494,7 @@
       <c r="D85" s="3">
         <v>7.36</v>
       </c>
-      <c r="E85" s="22" t="s">
+      <c r="E85" s="23" t="s">
         <v>165</v>
       </c>
       <c r="F85" s="5">
@@ -3277,7 +3514,7 @@
       <c r="D86" s="3">
         <v>30.52</v>
       </c>
-      <c r="E86" s="22" t="s">
+      <c r="E86" s="23" t="s">
         <v>166</v>
       </c>
       <c r="F86" s="5">
@@ -3297,7 +3534,7 @@
       <c r="D87" s="3">
         <v>6.05</v>
       </c>
-      <c r="E87" s="22" t="s">
+      <c r="E87" s="23" t="s">
         <v>167</v>
       </c>
       <c r="F87" s="5">
@@ -3317,7 +3554,7 @@
       <c r="D88" s="3">
         <v>4.67</v>
       </c>
-      <c r="E88" s="22" t="s">
+      <c r="E88" s="23" t="s">
         <v>168</v>
       </c>
       <c r="F88" s="5">
@@ -3337,7 +3574,7 @@
       <c r="D89" s="3">
         <v>15.58</v>
       </c>
-      <c r="E89" s="22" t="s">
+      <c r="E89" s="23" t="s">
         <v>169</v>
       </c>
       <c r="F89" s="5">
@@ -3357,7 +3594,7 @@
       <c r="D90" s="3">
         <v>18.63</v>
       </c>
-      <c r="E90" s="22" t="s">
+      <c r="E90" s="23" t="s">
         <v>170</v>
       </c>
       <c r="F90" s="5">
@@ -3377,7 +3614,7 @@
       <c r="D91" s="3">
         <v>10.99</v>
       </c>
-      <c r="E91" s="22" t="s">
+      <c r="E91" s="23" t="s">
         <v>171</v>
       </c>
       <c r="F91" s="5">
@@ -3397,7 +3634,7 @@
       <c r="D92" s="3">
         <v>22.97</v>
       </c>
-      <c r="E92" s="22" t="s">
+      <c r="E92" s="23" t="s">
         <v>172</v>
       </c>
       <c r="F92" s="5">
@@ -3417,7 +3654,7 @@
       <c r="D93" s="3">
         <v>18.150000000000002</v>
       </c>
-      <c r="E93" s="22" t="s">
+      <c r="E93" s="23" t="s">
         <v>173</v>
       </c>
       <c r="F93" s="5">
@@ -3437,7 +3674,7 @@
       <c r="D94" s="3">
         <v>12.83</v>
       </c>
-      <c r="E94" s="22" t="s">
+      <c r="E94" s="23" t="s">
         <v>174</v>
       </c>
       <c r="F94" s="5">
@@ -3457,7 +3694,7 @@
       <c r="D95" s="3">
         <v>42.25</v>
       </c>
-      <c r="E95" s="22" t="s">
+      <c r="E95" s="23" t="s">
         <v>175</v>
       </c>
       <c r="F95" s="5">
@@ -3477,7 +3714,7 @@
       <c r="D96" s="3">
         <v>17.38</v>
       </c>
-      <c r="E96" s="22" t="s">
+      <c r="E96" s="23" t="s">
         <v>176</v>
       </c>
       <c r="F96" s="5">
@@ -3497,7 +3734,7 @@
       <c r="D97" s="3">
         <v>27.18</v>
       </c>
-      <c r="E97" s="22" t="s">
+      <c r="E97" s="23" t="s">
         <v>177</v>
       </c>
       <c r="F97" s="5">
@@ -3517,7 +3754,7 @@
       <c r="D98" s="3">
         <v>34.51</v>
       </c>
-      <c r="E98" s="22" t="s">
+      <c r="E98" s="23" t="s">
         <v>178</v>
       </c>
       <c r="F98" s="5">
@@ -3537,7 +3774,7 @@
       <c r="D99" s="3">
         <v>42.57</v>
       </c>
-      <c r="E99" s="22" t="s">
+      <c r="E99" s="23" t="s">
         <v>179</v>
       </c>
       <c r="F99" s="5">
@@ -3557,7 +3794,7 @@
       <c r="D100" s="3">
         <v>21.68</v>
       </c>
-      <c r="E100" s="22" t="s">
+      <c r="E100" s="23" t="s">
         <v>180</v>
       </c>
       <c r="F100" s="5">
@@ -3577,7 +3814,7 @@
       <c r="D101" s="3">
         <v>24.78</v>
       </c>
-      <c r="E101" s="22" t="s">
+      <c r="E101" s="23" t="s">
         <v>181</v>
       </c>
       <c r="F101" s="5">
@@ -3597,7 +3834,7 @@
       <c r="D102" s="3">
         <v>16.63</v>
       </c>
-      <c r="E102" s="22" t="s">
+      <c r="E102" s="23" t="s">
         <v>182</v>
       </c>
       <c r="F102" s="5">
@@ -3617,7 +3854,7 @@
       <c r="D103" s="3">
         <v>19.14</v>
       </c>
-      <c r="E103" s="22" t="s">
+      <c r="E103" s="23" t="s">
         <v>183</v>
       </c>
       <c r="F103" s="5">
@@ -3637,7 +3874,7 @@
       <c r="D104" s="3">
         <v>33.01</v>
       </c>
-      <c r="E104" s="22" t="s">
+      <c r="E104" s="23" t="s">
         <v>184</v>
       </c>
       <c r="F104" s="5">
@@ -3657,7 +3894,7 @@
       <c r="D105" s="3">
         <v>28.75</v>
       </c>
-      <c r="E105" s="24" t="s">
+      <c r="E105" s="9" t="s">
         <v>26</v>
       </c>
       <c r="F105" s="5">
@@ -3677,7 +3914,7 @@
       <c r="D106" s="3">
         <v>58.82</v>
       </c>
-      <c r="E106" s="24" t="s">
+      <c r="E106" s="9" t="s">
         <v>27</v>
       </c>
       <c r="F106" s="5">
@@ -3697,7 +3934,7 @@
       <c r="D107" s="3">
         <v>23.490000000000002</v>
       </c>
-      <c r="E107" s="24" t="s">
+      <c r="E107" s="9" t="s">
         <v>28</v>
       </c>
       <c r="F107" s="5">
@@ -3717,7 +3954,7 @@
       <c r="D108" s="3">
         <v>59.9</v>
       </c>
-      <c r="E108" s="24" t="s">
+      <c r="E108" s="9" t="s">
         <v>29</v>
       </c>
       <c r="F108" s="5">
@@ -3726,812 +3963,1124 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="5"/>
-      <c r="B109" s="11"/>
+      <c r="B109" s="2" t="s">
+        <v>338</v>
+      </c>
       <c r="C109" s="5"/>
-      <c r="D109" s="14"/>
-      <c r="E109" s="15"/>
-      <c r="F109" s="13"/>
+      <c r="D109" s="3">
+        <v>10.89</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="F109" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="26"/>
-      <c r="B110" s="11"/>
+      <c r="A110" s="21"/>
+      <c r="B110" s="2" t="s">
+        <v>339</v>
+      </c>
       <c r="C110" s="5"/>
-      <c r="D110" s="14"/>
-      <c r="E110" s="15"/>
-      <c r="F110" s="13"/>
+      <c r="D110" s="3">
+        <v>20.63</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="F110" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="5"/>
-      <c r="B111" s="11"/>
+      <c r="B111" s="2" t="s">
+        <v>340</v>
+      </c>
       <c r="C111" s="5"/>
-      <c r="E111" s="12"/>
-      <c r="F111" s="5"/>
+      <c r="D111" s="3">
+        <v>35.6</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="F111" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="5"/>
-      <c r="B112" s="11"/>
+      <c r="B112" s="2" t="s">
+        <v>341</v>
+      </c>
       <c r="C112" s="5"/>
-      <c r="E112" s="12"/>
-      <c r="F112" s="5"/>
+      <c r="D112" s="3">
+        <v>30.21</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="F112" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="5"/>
-      <c r="B113" s="11"/>
+      <c r="B113" s="2" t="s">
+        <v>342</v>
+      </c>
       <c r="C113" s="5"/>
-      <c r="E113" s="12"/>
-      <c r="F113" s="5"/>
+      <c r="D113" s="3">
+        <v>33.06</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="F113" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="5"/>
-      <c r="B114" s="11"/>
+      <c r="B114" s="2" t="s">
+        <v>343</v>
+      </c>
       <c r="C114" s="5"/>
-      <c r="E114" s="12"/>
-      <c r="F114" s="5"/>
+      <c r="D114" s="3">
+        <v>17.82</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="F114" s="5">
+        <v>5</v>
+      </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="5"/>
-      <c r="B115" s="11"/>
+      <c r="B115" s="2" t="s">
+        <v>344</v>
+      </c>
       <c r="C115" s="5"/>
-      <c r="E115" s="12"/>
-      <c r="F115" s="5"/>
+      <c r="D115" s="3">
+        <v>14.33</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="F115" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="5"/>
-      <c r="B116" s="11"/>
+      <c r="B116" s="2" t="s">
+        <v>345</v>
+      </c>
       <c r="C116" s="5"/>
-      <c r="D116" s="14"/>
-      <c r="E116" s="15"/>
-      <c r="F116" s="13"/>
+      <c r="D116" s="3">
+        <v>14.33</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="F116" s="5">
+        <v>5</v>
+      </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="5"/>
-      <c r="B117" s="11"/>
+      <c r="B117" s="2" t="s">
+        <v>346</v>
+      </c>
       <c r="C117" s="5"/>
-      <c r="D117" s="14"/>
-      <c r="E117" s="15"/>
-      <c r="F117" s="13"/>
+      <c r="D117" s="3">
+        <v>14.33</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="F117" s="5">
+        <v>-1</v>
+      </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="5"/>
-      <c r="B118" s="11"/>
+      <c r="B118" s="2" t="s">
+        <v>347</v>
+      </c>
       <c r="C118" s="5"/>
-      <c r="D118" s="14"/>
-      <c r="E118" s="15"/>
-      <c r="F118" s="13"/>
+      <c r="D118" s="3">
+        <v>46.160000000000004</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="F118" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="5"/>
-      <c r="B119" s="11"/>
+      <c r="B119" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="C119" s="5"/>
-      <c r="D119" s="14"/>
-      <c r="E119" s="15"/>
-      <c r="F119" s="13"/>
+      <c r="D119" s="3">
+        <v>61.71</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="F119" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="5"/>
-      <c r="B120" s="16"/>
+      <c r="B120" s="2" t="s">
+        <v>377</v>
+      </c>
       <c r="C120" s="5"/>
-      <c r="E120" s="12"/>
-      <c r="F120" s="5"/>
+      <c r="D120" s="3">
+        <v>15.6</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="F120" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="5"/>
-      <c r="B121" s="11"/>
+      <c r="B121" s="2" t="s">
+        <v>378</v>
+      </c>
       <c r="C121" s="5"/>
-      <c r="D121" s="14"/>
-      <c r="E121" s="15"/>
-      <c r="F121" s="13"/>
+      <c r="D121" s="3">
+        <v>13.73</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F121" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="5"/>
-      <c r="B122" s="11"/>
+      <c r="B122" s="2" t="s">
+        <v>379</v>
+      </c>
       <c r="C122" s="5"/>
-      <c r="D122" s="14"/>
-      <c r="E122" s="15"/>
-      <c r="F122" s="13"/>
+      <c r="D122" s="3">
+        <v>13.74</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="F122" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="5"/>
-      <c r="B123" s="11"/>
+      <c r="B123" s="2" t="s">
+        <v>380</v>
+      </c>
       <c r="C123" s="5"/>
-      <c r="D123" s="14"/>
-      <c r="E123" s="15"/>
-      <c r="F123" s="13"/>
+      <c r="D123" s="3">
+        <v>16.670000000000002</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F123" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="5"/>
-      <c r="B124" s="11"/>
+      <c r="B124" s="2" t="s">
+        <v>381</v>
+      </c>
       <c r="C124" s="5"/>
-      <c r="D124" s="14"/>
-      <c r="E124" s="15"/>
-      <c r="F124" s="13"/>
+      <c r="D124" s="3">
+        <v>24.490000000000002</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="F124" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="5"/>
-      <c r="B125" s="11"/>
+      <c r="B125" s="2" t="s">
+        <v>382</v>
+      </c>
       <c r="C125" s="5"/>
-      <c r="D125" s="14"/>
-      <c r="E125" s="15"/>
-      <c r="F125" s="13"/>
+      <c r="D125" s="3">
+        <v>14.31</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="F125" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="5"/>
-      <c r="B126" s="11"/>
+      <c r="B126" s="2" t="s">
+        <v>383</v>
+      </c>
       <c r="C126" s="5"/>
-      <c r="D126" s="14"/>
-      <c r="E126" s="15"/>
-      <c r="F126" s="13"/>
+      <c r="D126" s="3">
+        <v>21.54</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="F126" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="5"/>
-      <c r="B127" s="11"/>
+      <c r="B127" s="2" t="s">
+        <v>384</v>
+      </c>
       <c r="C127" s="5"/>
-      <c r="D127" s="14"/>
-      <c r="E127" s="15"/>
-      <c r="F127" s="13"/>
+      <c r="D127" s="3">
+        <v>48.35</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="F127" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="5"/>
-      <c r="B128" s="11"/>
+      <c r="B128" s="2" t="s">
+        <v>385</v>
+      </c>
       <c r="C128" s="5"/>
-      <c r="D128" s="14"/>
-      <c r="E128" s="15"/>
-      <c r="F128" s="13"/>
+      <c r="D128" s="3">
+        <v>38.24</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="F128" s="5">
+        <v>5</v>
+      </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="5"/>
-      <c r="B129" s="11"/>
+      <c r="B129" s="2" t="s">
+        <v>386</v>
+      </c>
       <c r="C129" s="5"/>
-      <c r="D129" s="14"/>
-      <c r="E129" s="15"/>
-      <c r="F129" s="13"/>
+      <c r="D129" s="3">
+        <v>2.5300000000000002</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="F129" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="5"/>
-      <c r="B130" s="11"/>
+      <c r="B130" s="2" t="s">
+        <v>387</v>
+      </c>
       <c r="C130" s="5"/>
-      <c r="D130" s="14"/>
-      <c r="E130" s="15"/>
-      <c r="F130" s="13"/>
+      <c r="D130" s="3">
+        <v>16.7</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="F130" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="5"/>
-      <c r="B131" s="11"/>
+      <c r="B131" s="2" t="s">
+        <v>388</v>
+      </c>
       <c r="C131" s="5"/>
-      <c r="D131" s="14"/>
-      <c r="E131" s="15"/>
-      <c r="F131" s="13"/>
+      <c r="D131" s="3">
+        <v>19.490000000000002</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="F131" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="5"/>
-      <c r="B132" s="11"/>
+      <c r="B132" s="2" t="s">
+        <v>389</v>
+      </c>
       <c r="C132" s="5"/>
-      <c r="D132" s="14"/>
-      <c r="E132" s="15"/>
-      <c r="F132" s="13"/>
+      <c r="D132" s="3">
+        <v>14.96</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="F132" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="5"/>
-      <c r="B133" s="11"/>
+      <c r="B133" s="2" t="s">
+        <v>390</v>
+      </c>
       <c r="C133" s="5"/>
-      <c r="D133" s="14"/>
-      <c r="E133" s="15"/>
-      <c r="F133" s="13"/>
+      <c r="D133" s="3">
+        <v>36.78</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="F133" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="5"/>
-      <c r="B134" s="11"/>
+      <c r="B134" s="2" t="s">
+        <v>391</v>
+      </c>
       <c r="C134" s="5"/>
-      <c r="D134" s="14"/>
-      <c r="E134" s="15"/>
-      <c r="F134" s="13"/>
+      <c r="D134" s="3">
+        <v>21.6</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F134" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="5"/>
-      <c r="B135" s="11"/>
+      <c r="B135" s="2" t="s">
+        <v>392</v>
+      </c>
       <c r="C135" s="5"/>
-      <c r="D135" s="14"/>
-      <c r="E135" s="15"/>
-      <c r="F135" s="13"/>
+      <c r="D135" s="3">
+        <v>8.24</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="F135" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="5"/>
-      <c r="B136" s="11"/>
+      <c r="B136" s="2" t="s">
+        <v>393</v>
+      </c>
       <c r="C136" s="5"/>
-      <c r="D136" s="14"/>
-      <c r="E136" s="15"/>
-      <c r="F136" s="13"/>
+      <c r="D136" s="3">
+        <v>3.7</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="F136" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="5"/>
-      <c r="B137" s="11"/>
+      <c r="B137" s="2" t="s">
+        <v>394</v>
+      </c>
       <c r="C137" s="5"/>
-      <c r="D137" s="14"/>
-      <c r="E137" s="15"/>
-      <c r="F137" s="13"/>
+      <c r="D137" s="3">
+        <v>3.42</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="F137" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="5"/>
-      <c r="B138" s="11"/>
+      <c r="B138" s="2" t="s">
+        <v>395</v>
+      </c>
       <c r="C138" s="5"/>
-      <c r="D138" s="14"/>
-      <c r="E138" s="15"/>
-      <c r="F138" s="13"/>
+      <c r="D138" s="3">
+        <v>4.59</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="F138" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="5"/>
-      <c r="B139" s="11"/>
+      <c r="B139" s="2" t="s">
+        <v>396</v>
+      </c>
       <c r="C139" s="5"/>
-      <c r="D139" s="14"/>
-      <c r="E139" s="15"/>
-      <c r="F139" s="13"/>
+      <c r="D139" s="3">
+        <v>12.4</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="F139" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="5"/>
+      <c r="B140" s="2" t="s">
+        <v>397</v>
+      </c>
       <c r="C140" s="5"/>
-      <c r="E140" s="12"/>
-      <c r="F140" s="5"/>
+      <c r="D140" s="3">
+        <v>10.16</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="F140" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="5"/>
+      <c r="B141" s="2" t="s">
+        <v>398</v>
+      </c>
       <c r="C141" s="5"/>
-      <c r="E141" s="12"/>
-      <c r="F141" s="5"/>
+      <c r="D141" s="3">
+        <v>9.15</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F141" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="5"/>
+      <c r="B142" s="2" t="s">
+        <v>399</v>
+      </c>
       <c r="C142" s="5"/>
-      <c r="E142" s="12"/>
-      <c r="F142" s="5"/>
+      <c r="D142" s="3">
+        <v>11.69</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="F142" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="5"/>
+      <c r="B143" s="2" t="s">
+        <v>400</v>
+      </c>
       <c r="C143" s="5"/>
-      <c r="E143" s="12"/>
-      <c r="F143" s="5"/>
+      <c r="D143" s="3">
+        <v>6.32</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="F143" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="5"/>
+      <c r="B144" s="2" t="s">
+        <v>401</v>
+      </c>
       <c r="C144" s="5"/>
-      <c r="E144" s="12"/>
-      <c r="F144" s="5"/>
+      <c r="D144" s="3">
+        <v>4.96</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="F144" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="5"/>
+      <c r="B145" s="2" t="s">
+        <v>402</v>
+      </c>
       <c r="C145" s="5"/>
-      <c r="E145" s="12"/>
-      <c r="F145" s="5"/>
+      <c r="D145" s="3">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F145" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="5"/>
+      <c r="B146" s="2" t="s">
+        <v>403</v>
+      </c>
       <c r="C146" s="5"/>
-      <c r="E146" s="12"/>
-      <c r="F146" s="5"/>
+      <c r="D146" s="3">
+        <v>8.14</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="F146" s="5">
+        <v>9</v>
+      </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="5"/>
+      <c r="B147" s="2" t="s">
+        <v>404</v>
+      </c>
       <c r="C147" s="5"/>
-      <c r="E147" s="12"/>
-      <c r="F147" s="5"/>
+      <c r="D147" s="3">
+        <v>5</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="F147" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="5"/>
+      <c r="B148" s="2" t="s">
+        <v>407</v>
+      </c>
       <c r="C148" s="5"/>
-      <c r="E148" s="12"/>
-      <c r="F148" s="5"/>
+      <c r="D148" s="3">
+        <v>68.489999999999995</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="F148" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="5"/>
-      <c r="B149" s="11"/>
+      <c r="B149" s="2" t="s">
+        <v>408</v>
+      </c>
       <c r="C149" s="5"/>
-      <c r="D149" s="14"/>
-      <c r="E149" s="15"/>
-      <c r="F149" s="13"/>
+      <c r="D149" s="3">
+        <v>53.36</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="F149" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="5"/>
       <c r="B150" s="11"/>
       <c r="C150" s="5"/>
-      <c r="D150" s="14"/>
-      <c r="E150" s="15"/>
-      <c r="F150" s="13"/>
+      <c r="D150" s="13"/>
+      <c r="E150" s="11"/>
+      <c r="F150" s="12"/>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="5"/>
       <c r="B151" s="11"/>
       <c r="C151" s="5"/>
-      <c r="D151" s="14"/>
-      <c r="E151" s="15"/>
-      <c r="F151" s="13"/>
+      <c r="D151" s="13"/>
+      <c r="E151" s="11"/>
+      <c r="F151" s="12"/>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="5"/>
-      <c r="B152" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="C152" s="5"/>
-      <c r="D152" s="3">
-        <v>28.75</v>
-      </c>
-      <c r="E152" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="F152" s="5">
-        <v>7</v>
-      </c>
+      <c r="E152" s="2"/>
+      <c r="F152" s="5"/>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="5"/>
-      <c r="B153" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="C153" s="5"/>
-      <c r="D153" s="3">
-        <v>58.82</v>
-      </c>
-      <c r="E153" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F153" s="5">
-        <v>17</v>
-      </c>
+      <c r="E153" s="2"/>
+      <c r="F153" s="5"/>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="5"/>
-      <c r="B154" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="C154" s="5"/>
-      <c r="D154" s="3">
-        <v>23.490000000000002</v>
-      </c>
-      <c r="E154" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="F154" s="5">
-        <v>12</v>
-      </c>
+      <c r="E154" s="2"/>
+      <c r="F154" s="5"/>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="5"/>
-      <c r="B155" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="C155" s="5"/>
-      <c r="D155" s="3">
-        <v>59.9</v>
-      </c>
-      <c r="E155" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="F155" s="5">
-        <v>8</v>
-      </c>
+      <c r="E155" s="2"/>
+      <c r="F155" s="5"/>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="5"/>
       <c r="B156" s="11"/>
       <c r="C156" s="5"/>
-      <c r="D156" s="14"/>
-      <c r="E156" s="15"/>
-      <c r="F156" s="13"/>
+      <c r="D156" s="13"/>
+      <c r="E156" s="11"/>
+      <c r="F156" s="12"/>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="5"/>
       <c r="B157" s="11"/>
       <c r="C157" s="5"/>
-      <c r="D157" s="14"/>
-      <c r="E157" s="15"/>
-      <c r="F157" s="13"/>
+      <c r="D157" s="13"/>
+      <c r="E157" s="11"/>
+      <c r="F157" s="12"/>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="5"/>
       <c r="B158" s="11"/>
       <c r="C158" s="5"/>
-      <c r="D158" s="14"/>
-      <c r="E158" s="15"/>
-      <c r="F158" s="13"/>
+      <c r="D158" s="13"/>
+      <c r="E158" s="11"/>
+      <c r="F158" s="12"/>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="5"/>
       <c r="C159" s="5"/>
-      <c r="E159" s="12"/>
+      <c r="E159" s="2"/>
       <c r="F159" s="5"/>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="5"/>
       <c r="C160" s="5"/>
-      <c r="E160" s="12"/>
+      <c r="E160" s="2"/>
       <c r="F160" s="5"/>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="5"/>
       <c r="C161" s="5"/>
-      <c r="E161" s="12"/>
+      <c r="E161" s="2"/>
       <c r="F161" s="5"/>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="5"/>
       <c r="C162" s="5"/>
-      <c r="E162" s="12"/>
+      <c r="E162" s="2"/>
       <c r="F162" s="5"/>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="5"/>
       <c r="B163" s="11"/>
       <c r="C163" s="5"/>
-      <c r="E163" s="12"/>
+      <c r="E163" s="2"/>
       <c r="F163" s="5"/>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="5"/>
       <c r="B164" s="11"/>
       <c r="C164" s="5"/>
-      <c r="D164" s="14"/>
-      <c r="E164" s="15"/>
-      <c r="F164" s="13"/>
+      <c r="D164" s="13"/>
+      <c r="E164" s="11"/>
+      <c r="F164" s="12"/>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="5"/>
       <c r="B165" s="11"/>
       <c r="C165" s="5"/>
-      <c r="D165" s="14"/>
-      <c r="E165" s="15"/>
-      <c r="F165" s="13"/>
+      <c r="D165" s="13"/>
+      <c r="E165" s="11"/>
+      <c r="F165" s="12"/>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="5"/>
       <c r="B166" s="11"/>
       <c r="C166" s="5"/>
-      <c r="D166" s="14"/>
-      <c r="E166" s="15"/>
-      <c r="F166" s="13"/>
+      <c r="D166" s="13"/>
+      <c r="E166" s="11"/>
+      <c r="F166" s="12"/>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" s="5"/>
       <c r="B167" s="11"/>
       <c r="C167" s="5"/>
-      <c r="D167" s="14"/>
-      <c r="E167" s="15"/>
-      <c r="F167" s="13"/>
+      <c r="D167" s="13"/>
+      <c r="E167" s="11"/>
+      <c r="F167" s="12"/>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" s="5"/>
       <c r="B168" s="11"/>
       <c r="C168" s="5"/>
-      <c r="D168" s="14"/>
-      <c r="E168" s="15"/>
-      <c r="F168" s="13"/>
+      <c r="D168" s="13"/>
+      <c r="E168" s="11"/>
+      <c r="F168" s="12"/>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" s="5"/>
       <c r="B169" s="11"/>
       <c r="C169" s="5"/>
-      <c r="D169" s="14"/>
-      <c r="E169" s="15"/>
-      <c r="F169" s="13"/>
+      <c r="D169" s="13"/>
+      <c r="E169" s="11"/>
+      <c r="F169" s="12"/>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" s="5"/>
       <c r="B170" s="11"/>
       <c r="C170" s="5"/>
-      <c r="D170" s="14"/>
-      <c r="E170" s="15"/>
-      <c r="F170" s="13"/>
+      <c r="D170" s="13"/>
+      <c r="E170" s="11"/>
+      <c r="F170" s="12"/>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" s="5"/>
       <c r="B171" s="11"/>
       <c r="C171" s="5"/>
-      <c r="D171" s="14"/>
-      <c r="E171" s="15"/>
-      <c r="F171" s="13"/>
+      <c r="D171" s="13"/>
+      <c r="E171" s="11"/>
+      <c r="F171" s="12"/>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" s="5"/>
       <c r="B172" s="11"/>
       <c r="C172" s="5"/>
-      <c r="D172" s="14"/>
-      <c r="E172" s="15"/>
-      <c r="F172" s="13"/>
+      <c r="D172" s="13"/>
+      <c r="E172" s="11"/>
+      <c r="F172" s="12"/>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173" s="5"/>
       <c r="B173" s="11"/>
       <c r="C173" s="5"/>
-      <c r="D173" s="14"/>
-      <c r="E173" s="15"/>
-      <c r="F173" s="13"/>
+      <c r="D173" s="13"/>
+      <c r="E173" s="11"/>
+      <c r="F173" s="12"/>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174" s="5"/>
       <c r="B174" s="11"/>
       <c r="C174" s="5"/>
-      <c r="D174" s="14"/>
-      <c r="E174" s="15"/>
-      <c r="F174" s="13"/>
+      <c r="D174" s="13"/>
+      <c r="E174" s="11"/>
+      <c r="F174" s="12"/>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" s="5"/>
       <c r="B175" s="11"/>
       <c r="C175" s="5"/>
-      <c r="D175" s="14"/>
-      <c r="E175" s="15"/>
-      <c r="F175" s="13"/>
+      <c r="D175" s="13"/>
+      <c r="E175" s="11"/>
+      <c r="F175" s="12"/>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" s="5"/>
       <c r="B176" s="11"/>
       <c r="C176" s="5"/>
-      <c r="D176" s="14"/>
-      <c r="E176" s="15"/>
-      <c r="F176" s="13"/>
+      <c r="D176" s="13"/>
+      <c r="E176" s="11"/>
+      <c r="F176" s="12"/>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" s="5"/>
       <c r="B177" s="11"/>
       <c r="C177" s="5"/>
-      <c r="D177" s="14"/>
-      <c r="E177" s="15"/>
-      <c r="F177" s="13"/>
+      <c r="D177" s="13"/>
+      <c r="E177" s="11"/>
+      <c r="F177" s="12"/>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" s="5"/>
       <c r="B178" s="11"/>
       <c r="C178" s="5"/>
-      <c r="D178" s="14"/>
-      <c r="E178" s="15"/>
-      <c r="F178" s="13"/>
+      <c r="D178" s="13"/>
+      <c r="E178" s="11"/>
+      <c r="F178" s="12"/>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" s="5"/>
       <c r="B179" s="11"/>
       <c r="C179" s="5"/>
-      <c r="D179" s="14"/>
-      <c r="E179" s="15"/>
-      <c r="F179" s="13"/>
+      <c r="D179" s="13"/>
+      <c r="E179" s="11"/>
+      <c r="F179" s="12"/>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" s="5"/>
       <c r="C180" s="5"/>
-      <c r="E180" s="12"/>
+      <c r="E180" s="2"/>
       <c r="F180" s="5"/>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" s="5"/>
       <c r="C181" s="5"/>
-      <c r="E181" s="12"/>
+      <c r="E181" s="2"/>
       <c r="F181" s="5"/>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" s="5"/>
       <c r="B182" s="11"/>
       <c r="C182" s="5"/>
-      <c r="E182" s="12"/>
+      <c r="E182" s="2"/>
       <c r="F182" s="5"/>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" s="5"/>
       <c r="C183" s="5"/>
-      <c r="E183" s="12"/>
+      <c r="E183" s="2"/>
       <c r="F183" s="5"/>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" s="5"/>
       <c r="C184" s="5"/>
-      <c r="E184" s="12"/>
+      <c r="E184" s="2"/>
       <c r="F184" s="5"/>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" s="5"/>
       <c r="C185" s="5"/>
-      <c r="E185" s="12"/>
+      <c r="E185" s="2"/>
       <c r="F185" s="5"/>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186" s="5"/>
       <c r="C186" s="5"/>
-      <c r="E186" s="12"/>
+      <c r="E186" s="2"/>
       <c r="F186" s="5"/>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" s="5"/>
       <c r="C187" s="5"/>
-      <c r="E187" s="12"/>
+      <c r="E187" s="2"/>
       <c r="F187" s="5"/>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188" s="5"/>
       <c r="C188" s="5"/>
-      <c r="E188" s="12"/>
+      <c r="E188" s="2"/>
       <c r="F188" s="5"/>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" s="5"/>
       <c r="C189" s="5"/>
-      <c r="E189" s="12"/>
+      <c r="E189" s="2"/>
       <c r="F189" s="5"/>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" s="5"/>
       <c r="C190" s="5"/>
-      <c r="E190" s="12"/>
+      <c r="E190" s="2"/>
       <c r="F190" s="5"/>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" s="5"/>
       <c r="C191" s="5"/>
-      <c r="E191" s="12"/>
+      <c r="E191" s="2"/>
       <c r="F191" s="5"/>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" s="5"/>
       <c r="C192" s="5"/>
-      <c r="E192" s="12"/>
+      <c r="E192" s="2"/>
       <c r="F192" s="5"/>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" s="5"/>
       <c r="C193" s="5"/>
-      <c r="E193" s="12"/>
+      <c r="E193" s="2"/>
       <c r="F193" s="5"/>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194" s="5"/>
       <c r="C194" s="5"/>
-      <c r="E194" s="12"/>
+      <c r="E194" s="2"/>
       <c r="F194" s="5"/>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" s="5"/>
       <c r="C195" s="5"/>
-      <c r="E195" s="12"/>
+      <c r="E195" s="2"/>
       <c r="F195" s="5"/>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196" s="5"/>
       <c r="C196" s="5"/>
-      <c r="E196" s="12"/>
+      <c r="E196" s="2"/>
       <c r="F196" s="5"/>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" s="5"/>
       <c r="C197" s="5"/>
-      <c r="E197" s="12"/>
+      <c r="E197" s="2"/>
       <c r="F197" s="5"/>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198" s="5"/>
       <c r="C198" s="5"/>
-      <c r="E198" s="12"/>
+      <c r="E198" s="2"/>
       <c r="F198" s="5"/>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199" s="5"/>
       <c r="C199" s="5"/>
-      <c r="E199" s="12"/>
+      <c r="E199" s="2"/>
       <c r="F199" s="5"/>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200" s="5"/>
       <c r="C200" s="5"/>
-      <c r="E200" s="12"/>
+      <c r="E200" s="2"/>
       <c r="F200" s="5"/>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" s="5"/>
       <c r="C201" s="5"/>
-      <c r="E201" s="12"/>
+      <c r="E201" s="2"/>
       <c r="F201" s="5"/>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" s="5"/>
       <c r="C202" s="5"/>
-      <c r="E202" s="12"/>
+      <c r="E202" s="2"/>
       <c r="F202" s="5"/>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" s="5"/>
       <c r="C203" s="5"/>
-      <c r="E203" s="12"/>
+      <c r="E203" s="2"/>
       <c r="F203" s="5"/>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" s="5"/>
       <c r="C204" s="5"/>
-      <c r="E204" s="12"/>
+      <c r="E204" s="2"/>
       <c r="F204" s="5"/>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" s="5"/>
       <c r="C205" s="5"/>
-      <c r="E205" s="12"/>
+      <c r="E205" s="2"/>
       <c r="F205" s="5"/>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" s="5"/>
       <c r="C206" s="5"/>
-      <c r="E206" s="12"/>
+      <c r="E206" s="2"/>
       <c r="F206" s="5"/>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207" s="5"/>
       <c r="C207" s="5"/>
-      <c r="E207" s="12"/>
+      <c r="E207" s="2"/>
       <c r="F207" s="5"/>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208" s="5"/>
       <c r="C208" s="5"/>
-      <c r="E208" s="12"/>
+      <c r="E208" s="2"/>
       <c r="F208" s="5"/>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A209" s="5"/>
       <c r="C209" s="5"/>
-      <c r="E209" s="12"/>
+      <c r="E209" s="2"/>
       <c r="F209" s="5"/>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A210" s="5"/>
       <c r="C210" s="5"/>
-      <c r="E210" s="12"/>
+      <c r="E210" s="2"/>
       <c r="F210" s="5"/>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211" s="5"/>
       <c r="C211" s="5"/>
-      <c r="E211" s="12"/>
+      <c r="E211" s="2"/>
       <c r="F211" s="5"/>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A212" s="5"/>
       <c r="C212" s="5"/>
-      <c r="E212" s="12"/>
+      <c r="E212" s="2"/>
       <c r="F212" s="5"/>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A213" s="5"/>
       <c r="C213" s="5"/>
-      <c r="E213" s="12"/>
+      <c r="E213" s="2"/>
       <c r="F213" s="5"/>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A214" s="5"/>
       <c r="C214" s="5"/>
-      <c r="E214" s="12"/>
+      <c r="E214" s="2"/>
       <c r="F214" s="5"/>
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A215" s="5"/>
       <c r="C215" s="5"/>
-      <c r="E215" s="12"/>
+      <c r="E215" s="2"/>
       <c r="F215" s="5"/>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A216" s="5"/>
       <c r="B216" s="11"/>
       <c r="C216" s="5"/>
-      <c r="E216" s="12"/>
+      <c r="E216" s="2"/>
       <c r="F216" s="5"/>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A217" s="5"/>
       <c r="C217" s="5"/>
-      <c r="E217" s="12"/>
+      <c r="E217" s="2"/>
       <c r="F217" s="5"/>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A218" s="5"/>
       <c r="B218" s="11"/>
       <c r="C218" s="5"/>
-      <c r="E218" s="12"/>
+      <c r="E218" s="2"/>
       <c r="F218" s="5"/>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A219" s="5"/>
       <c r="C219" s="5"/>
-      <c r="E219" s="12"/>
+      <c r="E219" s="2"/>
       <c r="F219" s="5"/>
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>